<commit_message>
Pore space owner: pore_space field, PS01 flag, report section
Pore space follows the surface unless a deed reserves it, a separate pore
space conveyance exists, or a storage/sequestration agreement burdens it
(Myers-Woodward v. Underground Services Markham, Tex. 2025).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JbZzFNNZzsYuFmwDVFpT6y
</commit_message>
<xml_diff>
--- a/docs/TX_Surface_Fields_and_Rules.xlsx
+++ b/docs/TX_Surface_Fields_and_Rules.xlsx
@@ -665,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="15" min="1" max="1"/>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>homestead_indicators</t>
+          <t>pore_space</t>
         </is>
       </c>
       <c r="C20" s="22" t="inlineStr">
@@ -1365,14 +1365,22 @@
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>Homestead designation, spouse joinder or recitals</t>
+          <t>Any language about pore space, subsurface or underground storage space, geologic storage, storage reservoirs or salt caverns, or carbon dioxide (CO2) injection, storage or sequestration rights: grants, reservations, exceptions, leases, easements or options. Verbatim. Empty if none. A plain mineral reservation ('oil, gas and other minerals') is not pore space language: leave it in mineral_exception only</t>
         </is>
       </c>
       <c r="E20" s="23" t="n"/>
       <c r="F20" s="23" t="n"/>
-      <c r="G20" s="23" t="n"/>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>Added 2026-10-30: pore space owner</t>
+        </is>
+      </c>
       <c r="H20" s="23" t="n"/>
-      <c r="I20" s="24" t="n"/>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J20" s="23" t="inlineStr">
         <is>
           <t>Starter</t>
@@ -1387,17 +1395,17 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>easements</t>
+          <t>homestead_indicators</t>
         </is>
       </c>
       <c r="C21" s="22" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>Type (pipeline, road, utility, access, ROW), grantee, width, location description, term, assignability</t>
+          <t>Homestead designation, spouse joinder or recitals</t>
         </is>
       </c>
       <c r="E21" s="23" t="n"/>
@@ -1419,17 +1427,17 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>restrictions</t>
+          <t>easements</t>
         </is>
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>list</t>
         </is>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Deed restrictions, covenants and plat notes, verbatim</t>
+          <t>Type (pipeline, road, utility, access, ROW), grantee, width, location description, term, assignability</t>
         </is>
       </c>
       <c r="E22" s="23" t="n"/>
@@ -1451,17 +1459,17 @@
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>liens</t>
+          <t>restrictions</t>
         </is>
       </c>
       <c r="C23" s="22" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
         <is>
-          <t>Deed of trust, vendor's lien, judgment, tax or mechanic's lien, with holder, amount and release reference</t>
+          <t>Deed restrictions, covenants and plat notes, verbatim</t>
         </is>
       </c>
       <c r="E23" s="23" t="n"/>
@@ -1483,17 +1491,17 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>plat_reference</t>
+          <t>liens</t>
         </is>
       </c>
       <c r="C24" s="22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>list</t>
         </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>Subdivision, lot, block, plat cabinet and slide</t>
+          <t>Deed of trust, vendor's lien, judgment, tax or mechanic's lien, with holder, amount and release reference</t>
         </is>
       </c>
       <c r="E24" s="23" t="n"/>
@@ -1515,7 +1523,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>possession_notes</t>
+          <t>plat_reference</t>
         </is>
       </c>
       <c r="C25" s="22" t="inlineStr">
@@ -1525,7 +1533,7 @@
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>Affidavits of use and possession, adverse possession recitals</t>
+          <t>Subdivision, lot, block, plat cabinet and slide</t>
         </is>
       </c>
       <c r="E25" s="23" t="n"/>
@@ -1540,16 +1548,36 @@
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="16">
-      <c r="A26" s="23" t="n"/>
-      <c r="B26" s="23" t="n"/>
-      <c r="C26" s="23" t="n"/>
-      <c r="D26" s="23" t="n"/>
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>possession_notes</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Affidavits of use and possession, adverse possession recitals</t>
+        </is>
+      </c>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="23" t="n"/>
       <c r="G26" s="23" t="n"/>
       <c r="H26" s="23" t="n"/>
       <c r="I26" s="24" t="n"/>
-      <c r="J26" s="23" t="n"/>
+      <c r="J26" s="23" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="16">
       <c r="A27" s="23" t="n"/>
@@ -1838,6 +1866,18 @@
       <c r="H50" s="23" t="n"/>
       <c r="I50" s="24" t="n"/>
       <c r="J50" s="23" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="23" t="n"/>
+      <c r="B51" s="23" t="n"/>
+      <c r="C51" s="23" t="n"/>
+      <c r="D51" s="23" t="n"/>
+      <c r="E51" s="23" t="n"/>
+      <c r="F51" s="23" t="n"/>
+      <c r="G51" s="23" t="n"/>
+      <c r="H51" s="23" t="n"/>
+      <c r="I51" s="24" t="n"/>
+      <c r="J51" s="23" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J50"/>
@@ -1871,7 +1911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="1"/>
@@ -2440,17 +2480,49 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="16">
-      <c r="A19" s="23" t="n"/>
-      <c r="B19" s="23" t="n"/>
-      <c r="C19" s="23" t="n"/>
-      <c r="D19" s="23" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="23" t="n"/>
+    <row r="19" ht="23.85" customHeight="1" s="16">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>PS01</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Pore space language found: reservation or exception, separate conveyance of pore space, storage or sequestration lease/easement, or other mention. Pore space owner shown as the surface owner unless severed</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>Read the language; confirm the pore space owner and trace any reserved pore space forward</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Myers-Woodward, LLC v. Underground Services Markham, LLC (Tex. 2025): surface owner owns pore space absent agreement; pore space is not a mineral (confirm with counsel)</t>
+        </is>
+      </c>
       <c r="G19" s="23" t="n"/>
       <c r="H19" s="23" t="n"/>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="23" t="n"/>
+      <c r="I19" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="J19" s="23" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="16">
       <c r="A20" s="23" t="n"/>
@@ -2739,6 +2811,18 @@
       <c r="H43" s="23" t="n"/>
       <c r="I43" s="24" t="n"/>
       <c r="J43" s="23" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="23" t="n"/>
+      <c r="B44" s="23" t="n"/>
+      <c r="C44" s="23" t="n"/>
+      <c r="D44" s="23" t="n"/>
+      <c r="E44" s="23" t="n"/>
+      <c r="F44" s="23" t="n"/>
+      <c r="G44" s="23" t="n"/>
+      <c r="H44" s="23" t="n"/>
+      <c r="I44" s="24" t="n"/>
+      <c r="J44" s="23" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J43"/>

</xml_diff>

<commit_message>
Match SEG's final report layout (from the CCS.TX.SDY.0180 review)
- ROWs and Easements tab, same columns as the Runsheet; encumbrance sections point to it
- Active Material Encumbrances holds the major leases (SOLAR, WIND, CARBON, OGML, GRAZING) with TERM
- New 'term' extraction field
- Lease amendments/assignments and accommodation agreements stay in the Index
- Recorded-in county per instrument

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JbZzFNNZzsYuFmwDVFpT6y
</commit_message>
<xml_diff>
--- a/docs/TX_Surface_Fields_and_Rules.xlsx
+++ b/docs/TX_Surface_Fields_and_Rules.xlsx
@@ -665,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="15" min="1" max="1"/>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>homestead_indicators</t>
+          <t>term</t>
         </is>
       </c>
       <c r="C21" s="22" t="inlineStr">
@@ -1405,14 +1405,22 @@
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>Homestead designation, spouse joinder or recitals</t>
+          <t>The term of a lease, easement or timber deed as written: primary term, renewals, extensions and options (e.g. 'thirty (30) years ... two renewal terms of five (5) years each'). Empty if none stated</t>
         </is>
       </c>
       <c r="E21" s="23" t="n"/>
       <c r="F21" s="23" t="n"/>
-      <c r="G21" s="23" t="n"/>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>Added 2026-10-30: TERM column on the Encumbrances sheet</t>
+        </is>
+      </c>
       <c r="H21" s="23" t="n"/>
-      <c r="I21" s="24" t="n"/>
+      <c r="I21" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J21" s="23" t="inlineStr">
         <is>
           <t>Starter</t>
@@ -1427,17 +1435,17 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>easements</t>
+          <t>homestead_indicators</t>
         </is>
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Type (pipeline, road, utility, access, ROW), grantee, width, location description, term, assignability</t>
+          <t>Homestead designation, spouse joinder or recitals</t>
         </is>
       </c>
       <c r="E22" s="23" t="n"/>
@@ -1459,17 +1467,17 @@
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>restrictions</t>
+          <t>easements</t>
         </is>
       </c>
       <c r="C23" s="22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>list</t>
         </is>
       </c>
       <c r="D23" s="22" t="inlineStr">
         <is>
-          <t>Deed restrictions, covenants and plat notes, verbatim</t>
+          <t>Type (pipeline, road, utility, access, ROW), grantee, width, location description, term, assignability</t>
         </is>
       </c>
       <c r="E23" s="23" t="n"/>
@@ -1491,17 +1499,17 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>liens</t>
+          <t>restrictions</t>
         </is>
       </c>
       <c r="C24" s="22" t="inlineStr">
         <is>
-          <t>list</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>Deed of trust, vendor's lien, judgment, tax or mechanic's lien, with holder, amount and release reference</t>
+          <t>Deed restrictions, covenants and plat notes, verbatim</t>
         </is>
       </c>
       <c r="E24" s="23" t="n"/>
@@ -1523,17 +1531,17 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>plat_reference</t>
+          <t>liens</t>
         </is>
       </c>
       <c r="C25" s="22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>list</t>
         </is>
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>Subdivision, lot, block, plat cabinet and slide</t>
+          <t>Deed of trust, vendor's lien, judgment, tax or mechanic's lien, with holder, amount and release reference</t>
         </is>
       </c>
       <c r="E25" s="23" t="n"/>
@@ -1555,7 +1563,7 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>possession_notes</t>
+          <t>plat_reference</t>
         </is>
       </c>
       <c r="C26" s="22" t="inlineStr">
@@ -1565,7 +1573,7 @@
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
-          <t>Affidavits of use and possession, adverse possession recitals</t>
+          <t>Subdivision, lot, block, plat cabinet and slide</t>
         </is>
       </c>
       <c r="E26" s="23" t="n"/>
@@ -1580,16 +1588,36 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="16">
-      <c r="A27" s="23" t="n"/>
-      <c r="B27" s="23" t="n"/>
-      <c r="C27" s="23" t="n"/>
-      <c r="D27" s="23" t="n"/>
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>possession_notes</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Affidavits of use and possession, adverse possession recitals</t>
+        </is>
+      </c>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
       <c r="G27" s="23" t="n"/>
       <c r="H27" s="23" t="n"/>
       <c r="I27" s="24" t="n"/>
-      <c r="J27" s="23" t="n"/>
+      <c r="J27" s="23" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="16">
       <c r="A28" s="23" t="n"/>
@@ -1878,6 +1906,18 @@
       <c r="H51" s="23" t="n"/>
       <c r="I51" s="24" t="n"/>
       <c r="J51" s="23" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="23" t="n"/>
+      <c r="B52" s="23" t="n"/>
+      <c r="C52" s="23" t="n"/>
+      <c r="D52" s="23" t="n"/>
+      <c r="E52" s="23" t="n"/>
+      <c r="F52" s="23" t="n"/>
+      <c r="G52" s="23" t="n"/>
+      <c r="H52" s="23" t="n"/>
+      <c r="I52" s="24" t="n"/>
+      <c r="J52" s="23" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J50"/>

</xml_diff>

<commit_message>
NUM01: catch misread numbers (shares must total 100%; words must match digits)
Adds a per-grantee share to party records, number-word parsing (fractions,
decimals, '&'), prompt guidance on copying numbers, and acreage/interest to
the low-confidence check. Tested on 1,099 word/digit pairs from CCS.TX.SDY.0180.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JbZzFNNZzsYuFmwDVFpT6y
</commit_message>
<xml_diff>
--- a/docs/TX_Surface_Fields_and_Rules.xlsx
+++ b/docs/TX_Surface_Fields_and_Rules.xlsx
@@ -2565,16 +2565,44 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="16">
-      <c r="A20" s="23" t="n"/>
-      <c r="B20" s="23" t="n"/>
-      <c r="C20" s="23" t="n"/>
-      <c r="D20" s="23" t="n"/>
-      <c r="E20" s="23" t="n"/>
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>NUM01</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>Possible misread number: grantee shares in an instrument don't total 100% of the interest conveyed, or a number written in words and digits disagrees (e.g. 'seven (1%)')</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>Look at the image of the page and correct the number</t>
+        </is>
+      </c>
       <c r="F20" s="23" t="n"/>
       <c r="G20" s="23" t="n"/>
       <c r="H20" s="23" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="23" t="n"/>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>Starter</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="16">
       <c r="A21" s="23" t="n"/>

</xml_diff>